<commit_message>
add mean accuracy information for each condition
</commit_message>
<xml_diff>
--- a/data/phenotype/preprocessed/ds006239/ds006239_multiple-run_accuracy.xlsx
+++ b/data/phenotype/preprocessed/ds006239/ds006239_multiple-run_accuracy.xlsx
@@ -1,26 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/isaac938/Library/CloudStorage/Box-Box/BDL/Member_Folders/Isaac/01_project/reading-PA-NVIQ/data/phenotype/preprocessed/ds006239/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chenh55\Box\BDL\Member_Folders\Isaac\01_project\reading-PA-NVIQ\data\phenotype\preprocessed\ds006239\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{633CE97A-2A92-3D46-836D-7AD4A22DDF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74BCCFF2-F159-4DAF-85E1-CD2310F16AB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18200" yWindow="1520" windowWidth="15420" windowHeight="17180" xr2:uid="{FDFECC5B-3E5C-3C41-8941-DE020C9F0537}"/>
+    <workbookView xWindow="6228" yWindow="2280" windowWidth="23040" windowHeight="12264" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ds006239_multiple-run_accuracy" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="32">
   <si>
     <t>unique_id</t>
   </si>
@@ -34,19 +39,40 @@
     <t>n_correct_O+P+</t>
   </si>
   <si>
+    <t>n_correct_O+P-</t>
+  </si>
+  <si>
+    <t>n_correct_O-P+</t>
+  </si>
+  <si>
     <t>n_correct_O-P-</t>
   </si>
   <si>
     <t>n_trial_O+P+</t>
   </si>
   <si>
+    <t>n_trial_O+P-</t>
+  </si>
+  <si>
+    <t>n_trial_O-P+</t>
+  </si>
+  <si>
     <t>n_trial_O-P-</t>
   </si>
   <si>
     <t>mean_acc_O+P+</t>
   </si>
   <si>
+    <t>mean_acc_O+P-</t>
+  </si>
+  <si>
+    <t>mean_acc_O-P+</t>
+  </si>
+  <si>
     <t>mean_acc_O-P-</t>
+  </si>
+  <si>
+    <t>n_trial</t>
   </si>
   <si>
     <t>ds006239_sub-1122</t>
@@ -103,23 +129,23 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="18"/>
       <color theme="3"/>
-      <name val="Aptos Display"/>
+      <name val="Calibri Light"/>
       <family val="2"/>
       <scheme val="major"/>
     </font>
@@ -127,7 +153,7 @@
       <b/>
       <sz val="15"/>
       <color theme="3"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -135,7 +161,7 @@
       <b/>
       <sz val="13"/>
       <color theme="3"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -143,96 +169,96 @@
       <b/>
       <sz val="11"/>
       <color theme="3"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FF006100"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FF9C0006"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FF9C5700"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FF3F3F76"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FF3F3F3F"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="0"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <i/>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FF7F7F7F"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="0"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -649,39 +675,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -733,7 +759,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -844,6 +870,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -852,13 +885,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -923,46 +949,22 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E375E9A0-BD6E-6547-81CA-5CA26B8C0233}">
-  <dimension ref="A1:I13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:P13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -990,356 +992,629 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D2">
         <v>12</v>
       </c>
       <c r="E2">
+        <v>10</v>
+      </c>
+      <c r="F2">
+        <v>10</v>
+      </c>
+      <c r="G2">
         <v>8</v>
       </c>
-      <c r="F2">
-        <v>12</v>
-      </c>
-      <c r="G2">
-        <v>12</v>
-      </c>
       <c r="H2">
+        <v>12</v>
+      </c>
+      <c r="I2">
+        <v>12</v>
+      </c>
+      <c r="J2">
+        <v>12</v>
+      </c>
+      <c r="K2">
+        <v>12</v>
+      </c>
+      <c r="L2">
         <v>1</v>
       </c>
-      <c r="I2">
+      <c r="M2">
+        <v>0.83299999999999996</v>
+      </c>
+      <c r="N2">
+        <v>0.83299999999999996</v>
+      </c>
+      <c r="O2">
         <v>0.66700000000000004</v>
       </c>
+      <c r="P2">
+        <v>48</v>
+      </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3">
+        <v>12</v>
+      </c>
+      <c r="E3">
+        <v>8</v>
+      </c>
+      <c r="F3">
+        <v>10</v>
+      </c>
+      <c r="G3">
         <v>11</v>
       </c>
-      <c r="D3">
-        <v>12</v>
-      </c>
-      <c r="E3">
-        <v>11</v>
-      </c>
-      <c r="F3">
-        <v>12</v>
-      </c>
-      <c r="G3">
-        <v>12</v>
-      </c>
       <c r="H3">
+        <v>12</v>
+      </c>
+      <c r="I3">
+        <v>12</v>
+      </c>
+      <c r="J3">
+        <v>12</v>
+      </c>
+      <c r="K3">
+        <v>12</v>
+      </c>
+      <c r="L3">
         <v>1</v>
       </c>
-      <c r="I3">
+      <c r="M3">
+        <v>0.66700000000000004</v>
+      </c>
+      <c r="N3">
+        <v>0.83299999999999996</v>
+      </c>
+      <c r="O3">
         <v>0.91700000000000004</v>
       </c>
+      <c r="P3">
+        <v>48</v>
+      </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D4">
         <v>10</v>
       </c>
       <c r="E4">
+        <v>6</v>
+      </c>
+      <c r="F4">
+        <v>10</v>
+      </c>
+      <c r="G4">
         <v>9</v>
       </c>
-      <c r="F4">
-        <v>12</v>
-      </c>
-      <c r="G4">
-        <v>12</v>
-      </c>
       <c r="H4">
+        <v>12</v>
+      </c>
+      <c r="I4">
+        <v>12</v>
+      </c>
+      <c r="J4">
+        <v>12</v>
+      </c>
+      <c r="K4">
+        <v>12</v>
+      </c>
+      <c r="L4">
         <v>0.83299999999999996</v>
       </c>
-      <c r="I4">
+      <c r="M4">
+        <v>0.5</v>
+      </c>
+      <c r="N4">
+        <v>0.83299999999999996</v>
+      </c>
+      <c r="O4">
         <v>0.75</v>
       </c>
+      <c r="P4">
+        <v>48</v>
+      </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D5">
         <v>10</v>
       </c>
       <c r="E5">
+        <v>8</v>
+      </c>
+      <c r="F5">
+        <v>12</v>
+      </c>
+      <c r="G5">
         <v>10</v>
       </c>
-      <c r="F5">
-        <v>12</v>
-      </c>
-      <c r="G5">
-        <v>12</v>
-      </c>
       <c r="H5">
+        <v>12</v>
+      </c>
+      <c r="I5">
+        <v>12</v>
+      </c>
+      <c r="J5">
+        <v>12</v>
+      </c>
+      <c r="K5">
+        <v>12</v>
+      </c>
+      <c r="L5">
         <v>0.83299999999999996</v>
       </c>
-      <c r="I5">
+      <c r="M5">
+        <v>0.66700000000000004</v>
+      </c>
+      <c r="N5">
+        <v>1</v>
+      </c>
+      <c r="O5">
         <v>0.83299999999999996</v>
       </c>
+      <c r="P5">
+        <v>48</v>
+      </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D6">
         <v>7</v>
       </c>
       <c r="E6">
+        <v>6</v>
+      </c>
+      <c r="F6">
+        <v>10</v>
+      </c>
+      <c r="G6">
         <v>8</v>
       </c>
-      <c r="F6">
-        <v>12</v>
-      </c>
-      <c r="G6">
-        <v>12</v>
-      </c>
       <c r="H6">
+        <v>12</v>
+      </c>
+      <c r="I6">
+        <v>12</v>
+      </c>
+      <c r="J6">
+        <v>12</v>
+      </c>
+      <c r="K6">
+        <v>12</v>
+      </c>
+      <c r="L6">
         <v>0.58299999999999996</v>
       </c>
-      <c r="I6">
+      <c r="M6">
+        <v>0.5</v>
+      </c>
+      <c r="N6">
+        <v>0.83299999999999996</v>
+      </c>
+      <c r="O6">
         <v>0.66700000000000004</v>
       </c>
+      <c r="P6">
+        <v>48</v>
+      </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
         <v>18</v>
-      </c>
-      <c r="C7" t="s">
-        <v>11</v>
       </c>
       <c r="D7">
         <v>10</v>
       </c>
       <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7">
+        <v>8</v>
+      </c>
+      <c r="G7">
         <v>10</v>
       </c>
-      <c r="F7">
-        <v>12</v>
-      </c>
-      <c r="G7">
-        <v>12</v>
-      </c>
       <c r="H7">
+        <v>12</v>
+      </c>
+      <c r="I7">
+        <v>12</v>
+      </c>
+      <c r="J7">
+        <v>12</v>
+      </c>
+      <c r="K7">
+        <v>12</v>
+      </c>
+      <c r="L7">
         <v>0.83299999999999996</v>
       </c>
-      <c r="I7">
+      <c r="M7">
+        <v>0.5</v>
+      </c>
+      <c r="N7">
+        <v>0.66700000000000004</v>
+      </c>
+      <c r="O7">
         <v>0.83299999999999996</v>
       </c>
+      <c r="P7">
+        <v>48</v>
+      </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D8">
         <v>10</v>
       </c>
       <c r="E8">
+        <v>6</v>
+      </c>
+      <c r="F8">
+        <v>8</v>
+      </c>
+      <c r="G8">
         <v>9</v>
       </c>
-      <c r="F8">
-        <v>12</v>
-      </c>
-      <c r="G8">
-        <v>12</v>
-      </c>
       <c r="H8">
+        <v>12</v>
+      </c>
+      <c r="I8">
+        <v>12</v>
+      </c>
+      <c r="J8">
+        <v>12</v>
+      </c>
+      <c r="K8">
+        <v>12</v>
+      </c>
+      <c r="L8">
         <v>0.83299999999999996</v>
       </c>
-      <c r="I8">
+      <c r="M8">
+        <v>0.5</v>
+      </c>
+      <c r="N8">
+        <v>0.66700000000000004</v>
+      </c>
+      <c r="O8">
         <v>0.75</v>
       </c>
+      <c r="P8">
+        <v>48</v>
+      </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" t="s">
         <v>19</v>
       </c>
-      <c r="B9" t="s">
-        <v>12</v>
-      </c>
       <c r="C9" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D9">
         <v>8</v>
       </c>
       <c r="E9">
+        <v>7</v>
+      </c>
+      <c r="F9">
+        <v>11</v>
+      </c>
+      <c r="G9">
         <v>9</v>
       </c>
-      <c r="F9">
-        <v>12</v>
-      </c>
-      <c r="G9">
-        <v>12</v>
-      </c>
       <c r="H9">
+        <v>12</v>
+      </c>
+      <c r="I9">
+        <v>12</v>
+      </c>
+      <c r="J9">
+        <v>12</v>
+      </c>
+      <c r="K9">
+        <v>12</v>
+      </c>
+      <c r="L9">
         <v>0.66700000000000004</v>
       </c>
-      <c r="I9">
+      <c r="M9">
+        <v>0.58299999999999996</v>
+      </c>
+      <c r="N9">
+        <v>0.91700000000000004</v>
+      </c>
+      <c r="O9">
         <v>0.75</v>
       </c>
+      <c r="P9">
+        <v>48</v>
+      </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D10">
         <v>5</v>
       </c>
       <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
         <v>6</v>
       </c>
-      <c r="F10">
-        <v>12</v>
-      </c>
       <c r="G10">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H10">
+        <v>12</v>
+      </c>
+      <c r="I10">
+        <v>12</v>
+      </c>
+      <c r="J10">
+        <v>12</v>
+      </c>
+      <c r="K10">
+        <v>12</v>
+      </c>
+      <c r="L10">
         <v>0.41699999999999998</v>
       </c>
-      <c r="I10">
+      <c r="M10">
+        <v>8.3000000000000004E-2</v>
+      </c>
+      <c r="N10">
         <v>0.5</v>
       </c>
+      <c r="O10">
+        <v>0.5</v>
+      </c>
+      <c r="P10">
+        <v>48</v>
+      </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" t="s">
         <v>20</v>
-      </c>
-      <c r="B11" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" t="s">
-        <v>13</v>
       </c>
       <c r="D11">
         <v>7</v>
       </c>
       <c r="E11">
+        <v>5</v>
+      </c>
+      <c r="F11">
+        <v>9</v>
+      </c>
+      <c r="G11">
         <v>6</v>
       </c>
-      <c r="F11">
-        <v>12</v>
-      </c>
-      <c r="G11">
-        <v>12</v>
-      </c>
       <c r="H11">
+        <v>12</v>
+      </c>
+      <c r="I11">
+        <v>12</v>
+      </c>
+      <c r="J11">
+        <v>12</v>
+      </c>
+      <c r="K11">
+        <v>12</v>
+      </c>
+      <c r="L11">
         <v>0.58299999999999996</v>
       </c>
-      <c r="I11">
+      <c r="M11">
+        <v>0.41699999999999998</v>
+      </c>
+      <c r="N11">
+        <v>0.75</v>
+      </c>
+      <c r="O11">
         <v>0.5</v>
       </c>
+      <c r="P11">
+        <v>48</v>
+      </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
         <v>18</v>
-      </c>
-      <c r="C12" t="s">
-        <v>11</v>
       </c>
       <c r="D12">
         <v>8</v>
       </c>
       <c r="E12">
+        <v>9</v>
+      </c>
+      <c r="F12">
+        <v>5</v>
+      </c>
+      <c r="G12">
         <v>11</v>
       </c>
-      <c r="F12">
-        <v>12</v>
-      </c>
-      <c r="G12">
-        <v>12</v>
-      </c>
       <c r="H12">
+        <v>12</v>
+      </c>
+      <c r="I12">
+        <v>12</v>
+      </c>
+      <c r="J12">
+        <v>12</v>
+      </c>
+      <c r="K12">
+        <v>12</v>
+      </c>
+      <c r="L12">
         <v>0.66700000000000004</v>
       </c>
-      <c r="I12">
+      <c r="M12">
+        <v>0.75</v>
+      </c>
+      <c r="N12">
+        <v>0.41699999999999998</v>
+      </c>
+      <c r="O12">
         <v>0.91700000000000004</v>
       </c>
+      <c r="P12">
+        <v>48</v>
+      </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C13" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D13">
         <v>5</v>
       </c>
       <c r="E13">
+        <v>10</v>
+      </c>
+      <c r="F13">
+        <v>5</v>
+      </c>
+      <c r="G13">
         <v>11</v>
       </c>
-      <c r="F13">
-        <v>12</v>
-      </c>
-      <c r="G13">
-        <v>12</v>
-      </c>
       <c r="H13">
+        <v>12</v>
+      </c>
+      <c r="I13">
+        <v>12</v>
+      </c>
+      <c r="J13">
+        <v>12</v>
+      </c>
+      <c r="K13">
+        <v>12</v>
+      </c>
+      <c r="L13">
         <v>0.41699999999999998</v>
       </c>
-      <c r="I13">
+      <c r="M13">
+        <v>0.83299999999999996</v>
+      </c>
+      <c r="N13">
+        <v>0.41699999999999998</v>
+      </c>
+      <c r="O13">
         <v>0.91700000000000004</v>
+      </c>
+      <c r="P13">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>